<commit_message>
updated decks and templates
</commit_message>
<xml_diff>
--- a/docs/output/proposed/offerings/assets/Agentic_AI_Readiness_Assessment_Client_Preparation_Checklists.xlsx
+++ b/docs/output/proposed/offerings/assets/Agentic_AI_Readiness_Assessment_Client_Preparation_Checklists.xlsx
@@ -554,7 +554,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Helps the assessment team understand how the workflow operates today.</t>
+          <t>For each workflow in scope, prepare a basic summary covering:</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -586,7 +586,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Helps the assessment team understand how the workflow operates today.</t>
+          <t>For each workflow in scope, prepare a basic summary covering:</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Helps the assessment team understand how the workflow operates today.</t>
+          <t>For each workflow in scope, prepare a basic summary covering:</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Helps the assessment team understand how the workflow operates today.</t>
+          <t>For each workflow in scope, prepare a basic summary covering:</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -682,7 +682,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Helps the assessment team understand how the workflow operates today.</t>
+          <t>For each workflow in scope, prepare a basic summary covering:</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -714,7 +714,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Helps the assessment team understand how the workflow operates today.</t>
+          <t>For each workflow in scope, prepare a basic summary covering:</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -746,7 +746,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Helps the assessment team understand how the workflow operates today.</t>
+          <t>For each workflow in scope, prepare a basic summary covering:</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -778,7 +778,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Helps the assessment team understand how the workflow operates today.</t>
+          <t>For each workflow in scope, prepare a basic summary covering:</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1034,7 +1034,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Provides existing materials that help ground the assessment.</t>
+          <t>Gather any of the following that already exist:</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Provides existing materials that help ground the assessment.</t>
+          <t>Gather any of the following that already exist:</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1098,7 +1098,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Provides existing materials that help ground the assessment.</t>
+          <t>Gather any of the following that already exist:</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1130,7 +1130,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Provides existing materials that help ground the assessment.</t>
+          <t>Gather any of the following that already exist:</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Provides existing materials that help ground the assessment.</t>
+          <t>Gather any of the following that already exist:</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1194,7 +1194,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Provides existing materials that help ground the assessment.</t>
+          <t>Gather any of the following that already exist:</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1226,7 +1226,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Provides existing materials that help ground the assessment.</t>
+          <t>Gather any of the following that already exist:</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Provides existing materials that help ground the assessment.</t>
+          <t>Gather any of the following that already exist:</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1290,7 +1290,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Clarifies system, tool, and access context for the workflow.</t>
+          <t>For each workflow, prepare a simple list of:</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Clarifies system, tool, and access context for the workflow.</t>
+          <t>For each workflow, prepare a simple list of:</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Clarifies system, tool, and access context for the workflow.</t>
+          <t>For each workflow, prepare a simple list of:</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Clarifies system, tool, and access context for the workflow.</t>
+          <t>For each workflow, prepare a simple list of:</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Clarifies system, tool, and access context for the workflow.</t>
+          <t>For each workflow, prepare a simple list of:</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1450,7 +1450,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Clarifies system, tool, and access context for the workflow.</t>
+          <t>For each workflow, prepare a simple list of:</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1482,7 +1482,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Highlights practical execution constraints that affect readiness.</t>
+          <t>Also note:</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1514,7 +1514,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Highlights practical execution constraints that affect readiness.</t>
+          <t>Also note:</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1546,7 +1546,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Highlights practical execution constraints that affect readiness.</t>
+          <t>Also note:</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Provides current performance signals for the workflow.</t>
+          <t>Where available, share current measures such as:</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Provides current performance signals for the workflow.</t>
+          <t>Where available, share current measures such as:</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1642,7 +1642,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Provides current performance signals for the workflow.</t>
+          <t>Where available, share current measures such as:</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1674,7 +1674,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Provides current performance signals for the workflow.</t>
+          <t>Where available, share current measures such as:</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1706,7 +1706,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Provides current performance signals for the workflow.</t>
+          <t>Where available, share current measures such as:</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1738,7 +1738,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Provides current performance signals for the workflow.</t>
+          <t>Where available, share current measures such as:</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1770,7 +1770,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Provides current performance signals for the workflow.</t>
+          <t>Where available, share current measures such as:</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1802,7 +1802,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Provides current performance signals for the workflow.</t>
+          <t>Where available, share current measures such as:</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1834,7 +1834,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Provides directional performance context when formal metrics are unavailable.</t>
+          <t>If hard metrics are not available, provide directional indications such as:</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1866,7 +1866,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Provides directional performance context when formal metrics are unavailable.</t>
+          <t>If hard metrics are not available, provide directional indications such as:</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1898,7 +1898,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Provides directional performance context when formal metrics are unavailable.</t>
+          <t>If hard metrics are not available, provide directional indications such as:</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1930,7 +1930,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Provides directional performance context when formal metrics are unavailable.</t>
+          <t>If hard metrics are not available, provide directional indications such as:</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1962,7 +1962,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Provides directional performance context when formal metrics are unavailable.</t>
+          <t>If hard metrics are not available, provide directional indications such as:</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Surfaces known governance, control, and risk requirements.</t>
+          <t>For each workflow, note any known requirements or constraints relating to:</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Surfaces known governance, control, and risk requirements.</t>
+          <t>For each workflow, note any known requirements or constraints relating to:</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -2058,7 +2058,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Surfaces known governance, control, and risk requirements.</t>
+          <t>For each workflow, note any known requirements or constraints relating to:</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -2090,7 +2090,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Surfaces known governance, control, and risk requirements.</t>
+          <t>For each workflow, note any known requirements or constraints relating to:</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -2122,7 +2122,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Surfaces known governance, control, and risk requirements.</t>
+          <t>For each workflow, note any known requirements or constraints relating to:</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2154,7 +2154,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Surfaces known governance, control, and risk requirements.</t>
+          <t>For each workflow, note any known requirements or constraints relating to:</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Surfaces known governance, control, and risk requirements.</t>
+          <t>For each workflow, note any known requirements or constraints relating to:</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2218,7 +2218,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Surfaces known governance, control, and risk requirements.</t>
+          <t>For each workflow, note any known requirements or constraints relating to:</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2250,7 +2250,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Clarifies current ownership and failure handling.</t>
+          <t>Also identify:</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2282,7 +2282,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Clarifies current ownership and failure handling.</t>
+          <t>Also identify:</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2314,7 +2314,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Clarifies current ownership and failure handling.</t>
+          <t>Also identify:</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2346,7 +2346,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Provides concrete examples to ground the assessment.</t>
+          <t>Prepare 2 to 5 representative examples per workflow where possible:</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2378,7 +2378,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Provides concrete examples to ground the assessment.</t>
+          <t>Prepare 2 to 5 representative examples per workflow where possible:</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -2410,7 +2410,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Provides concrete examples to ground the assessment.</t>
+          <t>Prepare 2 to 5 representative examples per workflow where possible:</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2442,7 +2442,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Captures the practical flow of representative cases.</t>
+          <t>For each example, provide:</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2474,7 +2474,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Captures the practical flow of representative cases.</t>
+          <t>For each example, provide:</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2506,7 +2506,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Captures the practical flow of representative cases.</t>
+          <t>For each example, provide:</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2538,7 +2538,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Captures the practical flow of representative cases.</t>
+          <t>For each example, provide:</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2910,7 +2910,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F88"/>
+  <autoFilter ref="A1:F1"/>
 </worksheet>
 </file>
 
@@ -3740,7 +3740,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Ensures the assessment includes the right stakeholders.</t>
+          <t>Prepare a fuller stakeholder list covering:</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -3772,7 +3772,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Ensures the assessment includes the right stakeholders.</t>
+          <t>Prepare a fuller stakeholder list covering:</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -3804,7 +3804,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Ensures the assessment includes the right stakeholders.</t>
+          <t>Prepare a fuller stakeholder list covering:</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -3836,7 +3836,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Ensures the assessment includes the right stakeholders.</t>
+          <t>Prepare a fuller stakeholder list covering:</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -3868,7 +3868,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Ensures the assessment includes the right stakeholders.</t>
+          <t>Prepare a fuller stakeholder list covering:</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -3900,7 +3900,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Ensures the assessment includes the right stakeholders.</t>
+          <t>Prepare a fuller stakeholder list covering:</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3932,7 +3932,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Ensures the assessment includes the right stakeholders.</t>
+          <t>Prepare a fuller stakeholder list covering:</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3964,7 +3964,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Ensures the assessment includes the right stakeholders.</t>
+          <t>Prepare a fuller stakeholder list covering:</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3996,7 +3996,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Ensures the assessment includes the right stakeholders.</t>
+          <t>Prepare a fuller stakeholder list covering:</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -4028,7 +4028,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Clarifies how each stakeholder contributes to the assessment.</t>
+          <t>For each stakeholder, note:</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -4060,7 +4060,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Clarifies how each stakeholder contributes to the assessment.</t>
+          <t>For each stakeholder, note:</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -4092,7 +4092,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Clarifies how each stakeholder contributes to the assessment.</t>
+          <t>For each stakeholder, note:</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -4124,7 +4124,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Clarifies how each stakeholder contributes to the assessment.</t>
+          <t>For each stakeholder, note:</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -4156,7 +4156,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Provides supporting evidence for the governance and control review.</t>
+          <t>Prepare any available material related to:</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -4188,7 +4188,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Provides supporting evidence for the governance and control review.</t>
+          <t>Prepare any available material related to:</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -4220,7 +4220,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Provides supporting evidence for the governance and control review.</t>
+          <t>Prepare any available material related to:</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -4252,7 +4252,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Provides supporting evidence for the governance and control review.</t>
+          <t>Prepare any available material related to:</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -4284,7 +4284,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Provides supporting evidence for the governance and control review.</t>
+          <t>Prepare any available material related to:</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -4316,7 +4316,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Provides supporting evidence for the governance and control review.</t>
+          <t>Prepare any available material related to:</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -4348,7 +4348,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Provides supporting evidence for the governance and control review.</t>
+          <t>Prepare any available material related to:</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -4380,7 +4380,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Provides supporting evidence for the governance and control review.</t>
+          <t>Prepare any available material related to:</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -4412,7 +4412,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Provides supporting evidence for the governance and control review.</t>
+          <t>Prepare any available material related to:</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -4444,7 +4444,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Helps the team understand current control and failure-response practices.</t>
+          <t>Also be ready to explain:</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -4476,7 +4476,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Helps the team understand current control and failure-response practices.</t>
+          <t>Also be ready to explain:</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -4508,7 +4508,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Helps the team understand current control and failure-response practices.</t>
+          <t>Also be ready to explain:</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -4540,7 +4540,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Helps the team understand current control and failure-response practices.</t>
+          <t>Also be ready to explain:</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -4572,7 +4572,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Provides systems, data, and tooling context for the workflow.</t>
+          <t>For each workflow, provide:</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -4604,7 +4604,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Provides systems, data, and tooling context for the workflow.</t>
+          <t>For each workflow, provide:</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -4636,7 +4636,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Provides systems, data, and tooling context for the workflow.</t>
+          <t>For each workflow, provide:</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Provides systems, data, and tooling context for the workflow.</t>
+          <t>For each workflow, provide:</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -4700,7 +4700,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Provides systems, data, and tooling context for the workflow.</t>
+          <t>For each workflow, provide:</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -4732,7 +4732,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Provides systems, data, and tooling context for the workflow.</t>
+          <t>For each workflow, provide:</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -4764,7 +4764,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Provides systems, data, and tooling context for the workflow.</t>
+          <t>For each workflow, provide:</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -4796,7 +4796,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Provides systems, data, and tooling context for the workflow.</t>
+          <t>For each workflow, provide:</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -4828,7 +4828,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Highlights practical execution constraints that affect readiness.</t>
+          <t>Also note:</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -4860,7 +4860,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Highlights practical execution constraints that affect readiness.</t>
+          <t>Also note:</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -4892,7 +4892,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Highlights practical execution constraints that affect readiness.</t>
+          <t>Also note:</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Highlights practical execution constraints that affect readiness.</t>
+          <t>Also note:</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -4956,7 +4956,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Provides operational and quality signals for the assessment.</t>
+          <t>Where available, gather:</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -4988,7 +4988,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Provides operational and quality signals for the assessment.</t>
+          <t>Where available, gather:</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -5020,7 +5020,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Provides operational and quality signals for the assessment.</t>
+          <t>Where available, gather:</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -5052,7 +5052,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Provides operational and quality signals for the assessment.</t>
+          <t>Where available, gather:</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -5084,7 +5084,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Provides operational and quality signals for the assessment.</t>
+          <t>Where available, gather:</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -5116,7 +5116,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Provides operational and quality signals for the assessment.</t>
+          <t>Where available, gather:</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -5148,7 +5148,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Provides operational and quality signals for the assessment.</t>
+          <t>Where available, gather:</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -5180,7 +5180,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Provides operational and quality signals for the assessment.</t>
+          <t>Where available, gather:</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -5212,7 +5212,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Provides operational and quality signals for the assessment.</t>
+          <t>Where available, gather:</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -5244,7 +5244,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Provides operational and quality signals for the assessment.</t>
+          <t>Where available, gather:</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -5276,7 +5276,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Ensures the case set includes a useful range of workflow variants.</t>
+          <t>Where possible, include:</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -5308,7 +5308,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Ensures the case set includes a useful range of workflow variants.</t>
+          <t>Where possible, include:</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -5340,7 +5340,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Ensures the case set includes a useful range of workflow variants.</t>
+          <t>Where possible, include:</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -5372,7 +5372,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Ensures the case set includes a useful range of workflow variants.</t>
+          <t>Where possible, include:</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -5404,7 +5404,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Ensures the case set includes a useful range of workflow variants.</t>
+          <t>Where possible, include:</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -5436,7 +5436,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Ensures the case set includes a useful range of workflow variants.</t>
+          <t>Where possible, include:</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -5916,7 +5916,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Shows the organization’s likely ability to support a pilot.</t>
+          <t>This should include:</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -5948,7 +5948,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Shows the organization’s likely ability to support a pilot.</t>
+          <t>This should include:</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -5980,7 +5980,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Shows the organization’s likely ability to support a pilot.</t>
+          <t>This should include:</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -6012,7 +6012,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Shows the organization’s likely ability to support a pilot.</t>
+          <t>This should include:</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -6044,7 +6044,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Shows the organization’s likely ability to support a pilot.</t>
+          <t>This should include:</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -6076,7 +6076,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Shows the organization’s likely ability to support a pilot.</t>
+          <t>This should include:</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -6108,7 +6108,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Shows the organization’s likely ability to support a pilot.</t>
+          <t>This should include:</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -6332,7 +6332,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Provides additional context that can strengthen the Detailed Assessment.</t>
+          <t>If available, the following can improve the quality of the Detailed Assessment:</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -6364,7 +6364,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Provides additional context that can strengthen the Detailed Assessment.</t>
+          <t>If available, the following can improve the quality of the Detailed Assessment:</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -6396,7 +6396,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Provides additional context that can strengthen the Detailed Assessment.</t>
+          <t>If available, the following can improve the quality of the Detailed Assessment:</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -6428,7 +6428,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Provides additional context that can strengthen the Detailed Assessment.</t>
+          <t>If available, the following can improve the quality of the Detailed Assessment:</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -6460,7 +6460,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Provides additional context that can strengthen the Detailed Assessment.</t>
+          <t>If available, the following can improve the quality of the Detailed Assessment:</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -6492,7 +6492,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Provides additional context that can strengthen the Detailed Assessment.</t>
+          <t>If available, the following can improve the quality of the Detailed Assessment:</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -6524,7 +6524,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Provides additional context that can strengthen the Detailed Assessment.</t>
+          <t>If available, the following can improve the quality of the Detailed Assessment:</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -6556,7 +6556,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Confirms the deeper assessment can begin without avoidable delays.</t>
+          <t>Confirms the minimum inputs are in place before the assessment starts.</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -6588,7 +6588,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Confirms the deeper assessment can begin without avoidable delays.</t>
+          <t>Confirms the minimum inputs are in place before the assessment starts.</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -6620,7 +6620,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Confirms the deeper assessment can begin without avoidable delays.</t>
+          <t>Confirms the minimum inputs are in place before the assessment starts.</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -6652,7 +6652,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Confirms the deeper assessment can begin without avoidable delays.</t>
+          <t>Confirms the minimum inputs are in place before the assessment starts.</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -6684,7 +6684,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Confirms the deeper assessment can begin without avoidable delays.</t>
+          <t>Confirms the minimum inputs are in place before the assessment starts.</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -6716,7 +6716,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Confirms the deeper assessment can begin without avoidable delays.</t>
+          <t>Confirms the minimum inputs are in place before the assessment starts.</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -6748,7 +6748,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Confirms the deeper assessment can begin without avoidable delays.</t>
+          <t>Confirms the minimum inputs are in place before the assessment starts.</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -6780,7 +6780,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Confirms the deeper assessment can begin without avoidable delays.</t>
+          <t>Confirms the minimum inputs are in place before the assessment starts.</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -6812,7 +6812,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Confirms the deeper assessment can begin without avoidable delays.</t>
+          <t>Confirms the minimum inputs are in place before the assessment starts.</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -6844,7 +6844,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Confirms the deeper assessment can begin without avoidable delays.</t>
+          <t>Confirms the minimum inputs are in place before the assessment starts.</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -6876,7 +6876,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Confirms the deeper assessment can begin without avoidable delays.</t>
+          <t>Confirms the minimum inputs are in place before the assessment starts.</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -6896,6 +6896,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F124"/>
+  <autoFilter ref="A1:F1"/>
 </worksheet>
 </file>
</xml_diff>